<commit_message>
ingesta: snapshot 2026-09-04 18:36 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-09-04/CORDOBA_SEP26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-09-04/CORDOBA_SEP26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA4A968-D492-4E46-A6E7-B72B7C8B7285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2332D1-6041-41FF-B573-C4AF8BE8C28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
@@ -9963,10 +9963,10 @@
                   <c:v>114.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.7</c:v>
+                  <c:v>5.7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1</c:v>
+                  <c:v>18.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>-1</c:v>
@@ -19925,9 +19925,11 @@
         <v>0</v>
       </c>
       <c r="F3" s="24">
-        <v>2</v>
-      </c>
-      <c r="G3" s="25"/>
+        <v>0</v>
+      </c>
+      <c r="G3" s="25">
+        <v>0</v>
+      </c>
       <c r="H3" s="25"/>
       <c r="I3" s="25"/>
       <c r="J3" s="25"/>
@@ -19958,7 +19960,7 @@
       <c r="AI3" s="34"/>
       <c r="AJ3" s="36">
         <f>SUM(E3:AI3)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AK3" s="30">
         <v>27.817857142857147</v>
@@ -19983,7 +19985,9 @@
       <c r="F4" s="24">
         <v>0</v>
       </c>
-      <c r="G4" s="25"/>
+      <c r="G4" s="25">
+        <v>0</v>
+      </c>
       <c r="H4" s="25"/>
       <c r="I4" s="25"/>
       <c r="J4" s="25"/>
@@ -20039,7 +20043,9 @@
       <c r="F5" s="24">
         <v>0</v>
       </c>
-      <c r="G5" s="25"/>
+      <c r="G5" s="25">
+        <v>4.0999999999999996</v>
+      </c>
       <c r="H5" s="25"/>
       <c r="I5" s="25"/>
       <c r="J5" s="25"/>
@@ -20070,7 +20076,7 @@
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
         <f t="shared" si="0"/>
-        <v>65.099999999999994</v>
+        <v>69.199999999999989</v>
       </c>
       <c r="AK5" s="30">
         <v>40.986206896551728</v>
@@ -20095,7 +20101,9 @@
       <c r="F6" s="24">
         <v>0</v>
       </c>
-      <c r="G6" s="25"/>
+      <c r="G6" s="25">
+        <v>13.4</v>
+      </c>
       <c r="H6" s="25"/>
       <c r="I6" s="25"/>
       <c r="J6" s="25"/>
@@ -20126,7 +20134,7 @@
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>38.700000000000003</v>
+        <v>52.1</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20146,9 +20154,7 @@
         <v>19</v>
       </c>
       <c r="E7" s="24"/>
-      <c r="F7" s="24">
-        <v>0</v>
-      </c>
+      <c r="F7" s="24"/>
       <c r="G7" s="25"/>
       <c r="H7" s="25"/>
       <c r="I7" s="25"/>
@@ -20254,8 +20260,12 @@
       <c r="E9" s="24">
         <v>1</v>
       </c>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
+      <c r="F9" s="24">
+        <v>0</v>
+      </c>
+      <c r="G9" s="25">
+        <v>0</v>
+      </c>
       <c r="H9" s="25"/>
       <c r="I9" s="25"/>
       <c r="J9" s="25"/>
@@ -20306,9 +20316,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="24"/>
-      <c r="F10" s="24">
-        <v>0</v>
-      </c>
+      <c r="F10" s="24"/>
       <c r="G10" s="25"/>
       <c r="H10" s="25"/>
       <c r="I10" s="25"/>
@@ -20360,8 +20368,12 @@
       <c r="E11" s="24">
         <v>0</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="25"/>
+      <c r="F11" s="24">
+        <v>0.2</v>
+      </c>
+      <c r="G11" s="25">
+        <v>0.1</v>
+      </c>
       <c r="H11" s="25"/>
       <c r="I11" s="25"/>
       <c r="J11" s="25"/>
@@ -20392,7 +20404,7 @@
       <c r="AI11" s="34"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="AK11" s="30">
         <v>19.188461538461539</v>
@@ -20415,9 +20427,11 @@
         <v>1.5</v>
       </c>
       <c r="F12" s="24">
-        <v>0.2</v>
-      </c>
-      <c r="G12" s="25"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="25">
+        <v>0</v>
+      </c>
       <c r="H12" s="25"/>
       <c r="I12" s="25"/>
       <c r="J12" s="25"/>
@@ -20448,7 +20462,7 @@
       <c r="AI12" s="34"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="AK12" s="30">
         <v>34.724137931034484</v>
@@ -20471,9 +20485,11 @@
         <v>8</v>
       </c>
       <c r="F13" s="24">
-        <v>0</v>
-      </c>
-      <c r="G13" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="G13" s="25">
+        <v>0</v>
+      </c>
       <c r="H13" s="25"/>
       <c r="I13" s="25"/>
       <c r="J13" s="25"/>
@@ -20504,7 +20520,7 @@
       <c r="AI13" s="34"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK13" s="30"/>
     </row>
@@ -20525,9 +20541,11 @@
         <v>0</v>
       </c>
       <c r="F14" s="24">
-        <v>1</v>
-      </c>
-      <c r="G14" s="25"/>
+        <v>3.5</v>
+      </c>
+      <c r="G14" s="25">
+        <v>0</v>
+      </c>
       <c r="H14" s="25"/>
       <c r="I14" s="25"/>
       <c r="J14" s="25"/>
@@ -20558,7 +20576,7 @@
       <c r="AI14" s="34"/>
       <c r="AJ14" s="36">
         <f>SUM(E14:AI14)</f>
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="AK14" s="30">
         <v>36.1</v>
@@ -20581,9 +20599,11 @@
         <v>0.2</v>
       </c>
       <c r="F15" s="24">
-        <v>3.5</v>
-      </c>
-      <c r="G15" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="G15" s="25">
+        <v>1.2</v>
+      </c>
       <c r="H15" s="25"/>
       <c r="I15" s="25"/>
       <c r="J15" s="25"/>
@@ -20614,7 +20634,7 @@
       <c r="AI15" s="34"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="AK15" s="30">
         <v>60.46</v>
@@ -20634,9 +20654,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="32"/>
-      <c r="F16" s="32">
-        <v>1</v>
-      </c>
+      <c r="F16" s="32"/>
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
       <c r="I16" s="32"/>
@@ -20668,7 +20686,7 @@
       <c r="AI16" s="35"/>
       <c r="AJ16" s="36">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
@@ -20730,11 +20748,11 @@
       </c>
       <c r="F19" s="26">
         <f t="shared" ref="F19:AI19" si="1">IF(COUNT(F3:F17)&gt;0,SUM(F3:F17),-1)</f>
-        <v>7.7</v>
+        <v>5.7</v>
       </c>
       <c r="G19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>18.8</v>
       </c>
       <c r="H19" s="26">
         <f t="shared" si="1"/>

</xml_diff>